<commit_message>
- extract the file names of ss documents to create the tasks name for each of the file - create list of tasks to send to chatai - add new input inside first request prompt which is the tasks list to get the complexity and priority of the tasks
</commit_message>
<xml_diff>
--- a/Details_WBS.xlsx
+++ b/Details_WBS.xlsx
@@ -1201,7 +1201,7 @@
       </c>
       <c r="F2" s="37" t="n"/>
       <c r="G2" s="29" t="n">
-        <v>45663</v>
+        <v>45670</v>
       </c>
       <c r="H2" s="37" t="n"/>
     </row>
@@ -1211,13 +1211,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B3" s="32" t="inlineStr">
-        <is>
-          <t>This WBS incorporates the provided task breakdown and assigns tasks to team members based on complexity and skillset, aiming for a balanced workload. Jannatil Anwar Bin Jaharuddin, as the senior developer, is primarily assigned the hard tasks. The schedule aims to fully utilize the available time. The top three skills and experience with different platforms were considered when assigning tasks related to API integration, Data Validation/Extraction, and UI development.  The task durations are estimates and may be adjusted during project execution. While every effort was made to allocate tasks daily, minor adjustments might be necessary during the project. This version incorporates overlap between some team member's tasks to maintain continuous work.
-While every effort has been made to distribute the tasks equally and ensure daily work for every team member within the given timeframe, slight adjustments may be needed during project execution based on actual progress. Note:  Since task durations are estimated, the actual end date may differ from the planned end date.  If the project finishes earlier than the planned end date of 2025-03-07, a remark will be added below.
-This detailed WBS provides a structured approach to managing the WBS Enhancement project, facilitating better organization, tracking, and successful completion.  Because of the overlapping tasks and the short deadline, it assumes the team can handle multiple easy or easy/medium tasks concurrently.  This may need adjustment based on actual work velocity.</t>
-        </is>
-      </c>
+      <c r="B3" s="32" t="n"/>
       <c r="C3" s="38" t="n"/>
       <c r="D3" s="39" t="n"/>
       <c r="E3" s="34" t="inlineStr">
@@ -1357,7 +1351,7 @@
       </c>
       <c r="B6" s="21" t="inlineStr">
         <is>
-          <t>01/06/2025</t>
+          <t>01/13/2025</t>
         </is>
       </c>
       <c r="D6" s="26" t="inlineStr">
@@ -1879,11 +1873,13 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Develop UI for WBS Enhancement Screen** </t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="n">
-        <v/>
+          <t xml:space="preserve">WBS001_UI </t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jaharuddin, Jannatil Anwar Bin </t>
+        </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
@@ -1892,12 +1888,12 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>01/06/2025</t>
+          <t>01/13/2025</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>01/10/2025</t>
+          <t>01/17/2025</t>
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
@@ -1963,17 +1959,17 @@
     <row r="10" ht="12.6" customHeight="1">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.1 </t>
+          <t xml:space="preserve">2 </t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Implement layout for title, member skillset, and task details labels. </t>
+          <t xml:space="preserve">WBS002_UI </t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nur Ain Binti Mahamad Salleh </t>
+          <t xml:space="preserve">Jaharuddin, Jannatil Anwar Bin </t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
@@ -1983,12 +1979,12 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>01/06/2025</t>
+          <t>01/20/2025</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>01/06/2025</t>
+          <t>01/24/2025</t>
         </is>
       </c>
       <c r="G10" s="3" t="n"/>
@@ -2054,17 +2050,17 @@
     <row r="11" ht="12.6" customHeight="1">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.2 </t>
+          <t xml:space="preserve">3 </t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add input text fields for member skillset and task details. </t>
+          <t xml:space="preserve">WBS003_UI </t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nuramira Binti Ahmad Mahmud </t>
+          <t xml:space="preserve">Jaharuddin, Jannatil Anwar Bin </t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -2074,12 +2070,12 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>01/06/2025</t>
+          <t>01/27/2025</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>01/06/2025</t>
+          <t>01/31/2025</t>
         </is>
       </c>
       <c r="G11" s="3" t="n"/>
@@ -2145,17 +2141,17 @@
     <row r="12" ht="12.6" customHeight="1">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.3 </t>
+          <t xml:space="preserve">4 </t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Implement browse buttons for both input fields. </t>
+          <t xml:space="preserve">WBS001PRO001_CreateLoginFunction </t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Muhammad Izzun Mustaqim Bin Ismahdi </t>
+          <t xml:space="preserve">Jaharuddin, Jannatil Anwar Bin </t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
@@ -2165,12 +2161,12 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>01/07/2025</t>
+          <t>01/13/2025</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>01/07/2025</t>
+          <t>01/27/2025</t>
         </is>
       </c>
       <c r="G12" s="3" t="n"/>
@@ -2236,17 +2232,17 @@
     <row r="13" ht="12.6" customHeight="1">
       <c r="A13" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.4 </t>
+          <t xml:space="preserve">5 </t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Start and Cancel buttons. </t>
+          <t xml:space="preserve">WBS001PRO003_CreateRegisterFunction </t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jannatil Anwar Bin Jaharuddin </t>
+          <t xml:space="preserve">Jaharuddin, Jannatil Anwar Bin </t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -2256,12 +2252,12 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>01/07/2025</t>
+          <t>02/03/2025</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>01/07/2025</t>
+          <t>02/17/2025</t>
         </is>
       </c>
       <c r="G13" s="3" t="n"/>
@@ -2327,17 +2323,17 @@
     <row r="14" ht="12.6" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.5 </t>
+          <t xml:space="preserve">6 </t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Implement result label and text area. </t>
+          <t xml:space="preserve">WBS004_UI - Logout Confirmation Screen </t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nur Ain Binti Mahamad Salleh </t>
+          <t xml:space="preserve">Nuramira Binti Ahmad Mahmud </t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
@@ -2347,12 +2343,12 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>01/08/2025</t>
+          <t>01/13/2025</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>01/08/2025</t>
+          <t>01/15/2025</t>
         </is>
       </c>
       <c r="G14" s="3" t="n"/>
@@ -2418,17 +2414,17 @@
     <row r="15" ht="12.6" customHeight="1">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.6 </t>
+          <t xml:space="preserve">7 </t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add Download buttons (Download, Download 1, Download 2). </t>
+          <t xml:space="preserve">WBS001PRO002_CreateLogoutFunction </t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nuramira Binti Ahmad Mahmud </t>
+          <t xml:space="preserve">Muhammad Izzun Mustaqim Bin Ismahdi </t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -2438,12 +2434,12 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>01/08/2025</t>
+          <t>01/13/2025</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>01/08/2025</t>
+          <t>01/17/2025</t>
         </is>
       </c>
       <c r="G15" s="3" t="n"/>
@@ -2509,16 +2505,18 @@
     <row r="16" ht="12.6" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 </t>
+          <t xml:space="preserve">8 </t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Implement File Verification Logic** </t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="n">
-        <v/>
+          <t xml:space="preserve">WBS001PRO004_CreatePasswordResetFunction </t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Muhammad Izzun Mustaqim Bin Ismahdi </t>
+        </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
@@ -2527,12 +2525,12 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>01/13/2025</t>
+          <t>01/20/2025</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>01/15/2025</t>
+          <t>01/24/2025</t>
         </is>
       </c>
       <c r="G16" s="3" t="n"/>
@@ -2598,12 +2596,12 @@
     <row r="17" ht="12.6" customHeight="1">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.1 </t>
+          <t xml:space="preserve">9 </t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Check if uploaded file exists and is in the correct format. </t>
+          <t xml:space="preserve">Code Review - WBS001PRO001_CreateLoginFunction </t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -2618,12 +2616,12 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>01/13/2025</t>
+          <t>01/29/2025</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>01/13/2025</t>
+          <t>01/31/2025</t>
         </is>
       </c>
       <c r="G17" s="3" t="n"/>
@@ -2689,17 +2687,17 @@
     <row r="18" ht="12.6" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.2 </t>
+          <t xml:space="preserve">10 </t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handle file verification failures and display appropriate error messages. </t>
+          <t xml:space="preserve">Code Review - WBS001PRO003_CreateRegisterFunction </t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nuramira Binti Ahmad Mahmud </t>
+          <t xml:space="preserve">Muhammad Izzun Mustaqim Bin Ismahdi </t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
@@ -2709,12 +2707,12 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>01/14/2025</t>
+          <t>02/19/2025</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>01/14/2025</t>
+          <t>02/21/2025</t>
         </is>
       </c>
       <c r="G18" s="3" t="n"/>
@@ -2780,16 +2778,18 @@
     <row r="19" ht="12.6" customHeight="1">
       <c r="A19" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 </t>
+          <t xml:space="preserve">11 </t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Implement File Extraction Logic** </t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="n">
-        <v/>
+          <t xml:space="preserve">Testing - Login/Registration </t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nuramira Binti Ahmad Mahmud </t>
+        </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
@@ -2798,12 +2798,12 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>01/15/2025</t>
+          <t>01/29/2025</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>01/17/2025</t>
+          <t>02/01/2025</t>
         </is>
       </c>
       <c r="G19" s="3" t="n"/>
@@ -2869,17 +2869,17 @@
     <row r="20" ht="12.6" customHeight="1">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.1 </t>
+          <t xml:space="preserve">12 </t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Extract data from the uploaded file based on the template. </t>
+          <t xml:space="preserve">Testing - Logout functionality </t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jannatil Anwar Bin Jaharuddin </t>
+          <t xml:space="preserve">Nur Ain Binti Mahamad Salleh </t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
@@ -2889,12 +2889,12 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>01/15/2025</t>
+          <t>01/20/2025</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>01/16/2025</t>
+          <t>01/22/2025</t>
         </is>
       </c>
       <c r="G20" s="3" t="n"/>
@@ -2960,17 +2960,17 @@
     <row r="21" ht="12.6" customHeight="1">
       <c r="A21" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.2 </t>
+          <t xml:space="preserve">13 </t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handle extraction errors and display appropriate error messages. </t>
+          <t xml:space="preserve">Integration Testing - UI and Backend </t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Muhammad Izzun Mustaqim Bin Ismahdi </t>
+          <t xml:space="preserve">Nur Ain Binti Mahamad Salleh &amp; Nuramira Binti Ahmad Mahmud  </t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
@@ -2980,12 +2980,12 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>01/16/2025</t>
+          <t>02/03/2025</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>01/17/2025</t>
+          <t>02/07/2025</t>
         </is>
       </c>
       <c r="G21" s="3" t="n"/>
@@ -3051,16 +3051,18 @@
     <row r="22" ht="12.6" customHeight="1">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 </t>
+          <t xml:space="preserve">14 </t>
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Implement Data Validation Logic** </t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="n">
-        <v/>
+          <t xml:space="preserve">User Acceptance Testing (UAT) - All Features </t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All Team Members </t>
+        </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
@@ -3069,12 +3071,12 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>01/20/2025</t>
+          <t>02/19/2025</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>01/22/2025</t>
+          <t>03/01/2025</t>
         </is>
       </c>
       <c r="G22" s="3" t="n"/>
@@ -3140,17 +3142,17 @@
     <row r="23" ht="12.6" customHeight="1">
       <c r="A23" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.1 </t>
+          <t xml:space="preserve">15 </t>
         </is>
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Validate the extracted data against predefined rules. </t>
+          <t xml:space="preserve">Final Code Review and Refinements </t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nur Ain Binti Mahamad Salleh </t>
+          <t xml:space="preserve">Jaharuddin, Jannatil Anwar Bin </t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -3160,12 +3162,12 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>01/20/2025</t>
+          <t>03/04/2025</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>01/21/2025</t>
+          <t>03/10/2025</t>
         </is>
       </c>
       <c r="G23" s="3" t="n"/>
@@ -3231,17 +3233,17 @@
     <row r="24" ht="12.6" customHeight="1">
       <c r="A24" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.2 </t>
+          <t xml:space="preserve">16 </t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handle validation errors and display appropriate error messages. </t>
+          <t xml:space="preserve">Deployment Preparation </t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nuramira Binti Ahmad Mahmud </t>
+          <t xml:space="preserve">Jaharuddin, Jannatil Anwar Bin </t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
@@ -3251,12 +3253,12 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>01/21/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>01/22/2025</t>
+          <t>03/13/2025</t>
         </is>
       </c>
       <c r="G24" s="3" t="n"/>
@@ -3320,34 +3322,12 @@
       <c r="BM24" s="17" t="n"/>
     </row>
     <row r="25" ht="12.6" customHeight="1">
-      <c r="A25" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 </t>
-        </is>
-      </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Implement Read ChatAI API Key Functionality** </t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="n">
-        <v/>
-      </c>
-      <c r="D25" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>01/23/2025</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>01/24/2025</t>
-        </is>
-      </c>
+      <c r="A25" s="20" t="n"/>
+      <c r="B25" s="13" t="n"/>
+      <c r="C25" s="9" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
       <c r="G25" s="3" t="n"/>
       <c r="H25" s="3" t="n"/>
       <c r="I25" s="3" t="n"/>
@@ -3409,36 +3389,12 @@
       <c r="BM25" s="17" t="n"/>
     </row>
     <row r="26" ht="12.6" customHeight="1">
-      <c r="A26" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5.1 </t>
-        </is>
-      </c>
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Securely store and retrieve the ChatAI API Key. </t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jannatil Anwar Bin Jaharuddin </t>
-        </is>
-      </c>
-      <c r="D26" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>01/23/2025</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>01/24/2025</t>
-        </is>
-      </c>
+      <c r="A26" s="20" t="n"/>
+      <c r="B26" s="13" t="n"/>
+      <c r="C26" s="9" t="n"/>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
       <c r="G26" s="3" t="n"/>
       <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="n"/>
@@ -3500,34 +3456,12 @@
       <c r="BM26" s="17" t="n"/>
     </row>
     <row r="27" ht="12.6" customHeight="1">
-      <c r="A27" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 </t>
-        </is>
-      </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Implement Input Prompts Functionality** </t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="n">
-        <v/>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>01/27/2025</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>01/29/2025</t>
-        </is>
-      </c>
+      <c r="A27" s="20" t="n"/>
+      <c r="B27" s="13" t="n"/>
+      <c r="C27" s="9" t="n"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="3" t="n"/>
+      <c r="F27" s="3" t="n"/>
       <c r="G27" s="3" t="n"/>
       <c r="H27" s="3" t="n"/>
       <c r="I27" s="3" t="n"/>
@@ -3589,36 +3523,12 @@
       <c r="BM27" s="17" t="n"/>
     </row>
     <row r="28" ht="12.6" customHeight="1">
-      <c r="A28" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6.1 </t>
-        </is>
-      </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Generate prompts for ChatAI analysis based on extracted data. </t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Muhammad Izzun Mustaqim Bin Ismahdi </t>
-        </is>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>01/27/2025</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>01/29/2025</t>
-        </is>
-      </c>
+      <c r="A28" s="20" t="n"/>
+      <c r="B28" s="13" t="n"/>
+      <c r="C28" s="9" t="n"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n"/>
       <c r="G28" s="3" t="n"/>
       <c r="H28" s="3" t="n"/>
       <c r="I28" s="3" t="n"/>
@@ -3680,34 +3590,12 @@
       <c r="BM28" s="17" t="n"/>
     </row>
     <row r="29" ht="12.6" customHeight="1">
-      <c r="A29" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7 </t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Implement ChatAI Analysis** </t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="n">
-        <v/>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>01/29/2025</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>02/05/2025</t>
-        </is>
-      </c>
+      <c r="A29" s="15" t="n"/>
+      <c r="B29" s="9" t="n"/>
+      <c r="C29" s="9" t="n"/>
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="3" t="n"/>
+      <c r="F29" s="3" t="n"/>
       <c r="G29" s="3" t="n"/>
       <c r="H29" s="3" t="n"/>
       <c r="I29" s="3" t="n"/>
@@ -3769,36 +3657,12 @@
       <c r="BM29" s="17" t="n"/>
     </row>
     <row r="30" ht="12.6" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7.1 </t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Integrate with ChatAI API using the API key. </t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jannatil Anwar Bin Jaharuddin </t>
-        </is>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>01/29/2025</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>02/01/2025</t>
-        </is>
-      </c>
+      <c r="A30" s="15" t="n"/>
+      <c r="B30" s="9" t="n"/>
+      <c r="C30" s="9" t="n"/>
+      <c r="D30" s="12" t="n"/>
+      <c r="E30" s="3" t="n"/>
+      <c r="F30" s="3" t="n"/>
       <c r="G30" s="3" t="n"/>
       <c r="H30" s="3" t="n"/>
       <c r="I30" s="3" t="n"/>
@@ -3860,36 +3724,12 @@
       <c r="BM30" s="17" t="n"/>
     </row>
     <row r="31" ht="12.6" customHeight="1">
-      <c r="A31" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7.2 </t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Send prompts to ChatAI and receive analysis results. </t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Muhammad Izzun Mustaqim Bin Ismahdi </t>
-        </is>
-      </c>
-      <c r="D31" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>02/01/2025</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>02/03/2025</t>
-        </is>
-      </c>
+      <c r="A31" s="15" t="n"/>
+      <c r="B31" s="9" t="n"/>
+      <c r="C31" s="9" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="3" t="n"/>
+      <c r="F31" s="3" t="n"/>
       <c r="G31" s="3" t="n"/>
       <c r="H31" s="3" t="n"/>
       <c r="I31" s="3" t="n"/>
@@ -3951,36 +3791,12 @@
       <c r="BM31" s="17" t="n"/>
     </row>
     <row r="32" ht="12.6" customHeight="1">
-      <c r="A32" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7.3 </t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Handle ChatAI API errors and display appropriate error messages. </t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nuramira Binti Ahmad Mahmud </t>
-        </is>
-      </c>
-      <c r="D32" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>02/03/2025</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>02/05/2025</t>
-        </is>
-      </c>
+      <c r="A32" s="15" t="n"/>
+      <c r="B32" s="9" t="n"/>
+      <c r="C32" s="9" t="n"/>
+      <c r="D32" s="12" t="n"/>
+      <c r="E32" s="3" t="n"/>
+      <c r="F32" s="3" t="n"/>
       <c r="G32" s="3" t="n"/>
       <c r="H32" s="3" t="n"/>
       <c r="I32" s="3" t="n"/>
@@ -4042,34 +3858,12 @@
       <c r="BM32" s="17" t="n"/>
     </row>
     <row r="33" ht="12.6" customHeight="1">
-      <c r="A33" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8 </t>
-        </is>
-      </c>
-      <c r="B33" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Implement Result Validation Logic** </t>
-        </is>
-      </c>
-      <c r="C33" s="13" t="n">
-        <v/>
-      </c>
-      <c r="D33" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>02/06/2025</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>02/08/2025</t>
-        </is>
-      </c>
+      <c r="A33" s="18" t="n"/>
+      <c r="B33" s="19" t="n"/>
+      <c r="C33" s="13" t="n"/>
+      <c r="D33" s="12" t="n"/>
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="3" t="n"/>
       <c r="G33" s="3" t="n"/>
       <c r="H33" s="3" t="n"/>
       <c r="I33" s="3" t="n"/>
@@ -4131,36 +3925,12 @@
       <c r="BM33" s="17" t="n"/>
     </row>
     <row r="34" ht="12.6" customHeight="1">
-      <c r="A34" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8.1 </t>
-        </is>
-      </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Validate the ChatAI analysis results. </t>
-        </is>
-      </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nur Ain Binti Mahamad Salleh </t>
-        </is>
-      </c>
-      <c r="D34" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>02/06/2025</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>02/07/2025</t>
-        </is>
-      </c>
+      <c r="A34" s="20" t="n"/>
+      <c r="B34" s="13" t="n"/>
+      <c r="C34" s="9" t="n"/>
+      <c r="D34" s="12" t="n"/>
+      <c r="E34" s="3" t="n"/>
+      <c r="F34" s="3" t="n"/>
       <c r="G34" s="3" t="n"/>
       <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="n"/>
@@ -4222,36 +3992,12 @@
       <c r="BM34" s="17" t="n"/>
     </row>
     <row r="35" ht="12.6" customHeight="1">
-      <c r="A35" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8.2 </t>
-        </is>
-      </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Handle validation failures and display appropriate error messages. </t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jannatil Anwar Bin Jaharuddin </t>
-        </is>
-      </c>
-      <c r="D35" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>02/07/2025</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>02/08/2025</t>
-        </is>
-      </c>
+      <c r="A35" s="20" t="n"/>
+      <c r="B35" s="13" t="n"/>
+      <c r="C35" s="9" t="n"/>
+      <c r="D35" s="12" t="n"/>
+      <c r="E35" s="3" t="n"/>
+      <c r="F35" s="3" t="n"/>
       <c r="G35" s="3" t="n"/>
       <c r="H35" s="3" t="n"/>
       <c r="I35" s="3" t="n"/>
@@ -4313,34 +4059,12 @@
       <c r="BM35" s="17" t="n"/>
     </row>
     <row r="36" ht="12.6" customHeight="1">
-      <c r="A36" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9 </t>
-        </is>
-      </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Implement Result Generation and Display** </t>
-        </is>
-      </c>
-      <c r="C36" s="9" t="n">
-        <v/>
-      </c>
-      <c r="D36" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>02/10/2025</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>02/12/2025</t>
-        </is>
-      </c>
+      <c r="A36" s="20" t="n"/>
+      <c r="B36" s="13" t="n"/>
+      <c r="C36" s="9" t="n"/>
+      <c r="D36" s="12" t="n"/>
+      <c r="E36" s="3" t="n"/>
+      <c r="F36" s="3" t="n"/>
       <c r="G36" s="3" t="n"/>
       <c r="H36" s="3" t="n"/>
       <c r="I36" s="3" t="n"/>
@@ -4402,36 +4126,12 @@
       <c r="BM36" s="17" t="n"/>
     </row>
     <row r="37" ht="12.6" customHeight="1">
-      <c r="A37" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9.1 </t>
-        </is>
-      </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Format the ChatAI analysis results for display on the screen. </t>
-        </is>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Muhammad Izzun Mustaqim Bin Ismahdi </t>
-        </is>
-      </c>
-      <c r="D37" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>02/10/2025</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>02/11/2025</t>
-        </is>
-      </c>
+      <c r="A37" s="20" t="n"/>
+      <c r="B37" s="13" t="n"/>
+      <c r="C37" s="9" t="n"/>
+      <c r="D37" s="12" t="n"/>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
       <c r="G37" s="3" t="n"/>
       <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="n"/>
@@ -4493,36 +4193,12 @@
       <c r="BM37" s="17" t="n"/>
     </row>
     <row r="38" ht="12.6" customHeight="1">
-      <c r="A38" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9.2 </t>
-        </is>
-      </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Populate the result text area with the formatted results. </t>
-        </is>
-      </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nur Ain Binti Mahamad Salleh </t>
-        </is>
-      </c>
-      <c r="D38" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>02/11/2025</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>02/12/2025</t>
-        </is>
-      </c>
+      <c r="A38" s="20" t="n"/>
+      <c r="B38" s="13" t="n"/>
+      <c r="C38" s="9" t="n"/>
+      <c r="D38" s="12" t="n"/>
+      <c r="E38" s="3" t="n"/>
+      <c r="F38" s="3" t="n"/>
       <c r="G38" s="3" t="n"/>
       <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="n"/>
@@ -4584,34 +4260,12 @@
       <c r="BM38" s="17" t="n"/>
     </row>
     <row r="39" ht="12.6" customHeight="1">
-      <c r="A39" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10 </t>
-        </is>
-      </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">**Implement Download Functionality** </t>
-        </is>
-      </c>
-      <c r="C39" s="9" t="n">
-        <v/>
-      </c>
-      <c r="D39" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>02/12/2025</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>02/14/2025</t>
-        </is>
-      </c>
+      <c r="A39" s="20" t="n"/>
+      <c r="B39" s="13" t="n"/>
+      <c r="C39" s="9" t="n"/>
+      <c r="D39" s="12" t="n"/>
+      <c r="E39" s="3" t="n"/>
+      <c r="F39" s="3" t="n"/>
       <c r="G39" s="3" t="n"/>
       <c r="H39" s="3" t="n"/>
       <c r="I39" s="3" t="n"/>
@@ -4673,36 +4327,12 @@
       <c r="BM39" s="17" t="n"/>
     </row>
     <row r="40" ht="12.6" customHeight="1">
-      <c r="A40" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10.1 </t>
-        </is>
-      </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enable downloading of different result formats (based on Download buttons). </t>
-        </is>
-      </c>
-      <c r="C40" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nuramira Binti Ahmad Mahmud </t>
-        </is>
-      </c>
-      <c r="D40" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">To do </t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>02/12/2025</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>02/14/2025</t>
-        </is>
-      </c>
+      <c r="A40" s="20" t="n"/>
+      <c r="B40" s="13" t="n"/>
+      <c r="C40" s="9" t="n"/>
+      <c r="D40" s="12" t="n"/>
+      <c r="E40" s="3" t="n"/>
+      <c r="F40" s="3" t="n"/>
       <c r="G40" s="3" t="n"/>
       <c r="H40" s="3" t="n"/>
       <c r="I40" s="3" t="n"/>

</xml_diff>